<commit_message>
add demo excel files
</commit_message>
<xml_diff>
--- a/data/documents.xlsx
+++ b/data/documents.xlsx
@@ -19,34 +19,34 @@
     <t>Expiration Date</t>
   </si>
   <si>
-    <t xml:space="preserve">2026-02-02 РЕГЛАМЕНТ ЗАКЛЮЧЕНИЯ ПРЯМОГО МЕЖДУНАРОДНОГО КОНТРАКТА </t>
-  </si>
-  <si>
-    <t>2025-11-17 РЕГЛАМЕНТ ПО ОФОРМЛЕНИЮ СОТРУДНИКОВ ПО ТК РФ</t>
-  </si>
-  <si>
-    <t>2025-03-25 РЕГЛАМЕНТ ПО СБОРУ ДОКУМЕНТОВ ОТ КАНДИДАТА НА  ВАКАНТНУЮ ДОЛЖНОСТЬ И ОБНОВЛЕНИЯ ДОКУМЕНТОВ СОТРУДНИКА</t>
-  </si>
-  <si>
-    <t>2026-02-02 РЕГЛАМЕНТ ПО ПОДГОТОВКЕ И ПОДПИСАНИИ ДОКУМЕНТОВ ПРИ ПЕРЕХОДЕ СТАЖЕРА В ШТАТНОГО СОТРУДНИКА</t>
-  </si>
-  <si>
-    <t>2025-08-18 РЕГЛАМЕНТ РАБОТЫ С ПРИЗЫВНИКАМИ</t>
-  </si>
-  <si>
-    <t>2026-01-15: ИНСТРУКЦИЯ СООТВЕТСТВИЯ ГРЕЙДОВ ДОЛЖНОСТЯМ В ШТАТНОМ РАСПИСАНИИ</t>
-  </si>
-  <si>
-    <t>2026-05-15 РЕГЛАМЕНТ ПО РАСТОРЖЕНИЮ ДОГОВОРОВ</t>
-  </si>
-  <si>
-    <t>2026-05-08 РЕГЛАМЕНТ ВЗАИМОДЕЙСТВИЯ С САМОЗАНЯТЫМ</t>
-  </si>
-  <si>
-    <t>2026-03-27: РЕГЛАМЕНТ ПО ОБНОВЛЕНИЮ ШТАТНОГО РАСПИСАНИЯ</t>
-  </si>
-  <si>
-    <t>2026-02-03: ИНСТРУКЦИЯ ЗАПОЛНЕНИЯ ОТЧЕТА РЕВИЗИЯ ШТАТНОГО РАСПИСАНИЯ</t>
+    <t xml:space="preserve">РЕГЛАМЕНТ ЗАКЛЮЧЕНИЯ КОНТРАКТА </t>
+  </si>
+  <si>
+    <t>РЕГЛАМЕНТ ПО ОФОРМЛЕНИЮ СОТРУДНИКОВ</t>
+  </si>
+  <si>
+    <t>РЕГЛАМЕНТ ПО СБОРУ ДОКУМЕНТОВ ОТ КАНДИДАТА</t>
+  </si>
+  <si>
+    <t>РЕГЛАМЕНТ ПО ПОДГОТОВКЕ ДОКУМЕНТОВ ПРИ ПЕРЕХОДЕ СТАЖЕРА В ШТАТНОГО СОТРУДНИКА</t>
+  </si>
+  <si>
+    <t>РЕГЛАМЕНТ РАБОТЫ С ПРИЗЫВНИКАМИ</t>
+  </si>
+  <si>
+    <t>ИНСТРУКЦИЯ СООТВЕТСТВИЯ ГРЕЙДОВ</t>
+  </si>
+  <si>
+    <t>2РЕГЛАМЕНТ ПО РАСТОРЖЕНИЮ ДОГОВОРОВ</t>
+  </si>
+  <si>
+    <t>РЕГЛАМЕНТ ВЗАИМОДЕЙСТВИЯ С САМОЗАНЯТЫМ</t>
+  </si>
+  <si>
+    <t>РЕГЛАМЕНТ ПО ОБНОВЛЕНИЮ ШТАТНОГО РАСПИСАНИЯ</t>
+  </si>
+  <si>
+    <t>ИНСТРУКЦИЯ ЗАПОЛНЕНИЯ ОТЧЕТА РЕВИЗИЯ ШТАТНОГО РАСПИСАНИЯ</t>
   </si>
 </sst>
 </file>
@@ -55,9 +55,9 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:a15="http://schemas.microsoft.com/office/drawing/2012/main" xmlns:asvg="http://schemas.microsoft.com/office/drawing/2016/SVG/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:co="http://ncloudtech.com" xmlns:co-ooxml="http://ncloudtech.com/ooxml" xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:o="urn:schemas-microsoft-com:office:office" xmlns:p="http://schemas.openxmlformats.org/presentationml/2006/main" xmlns:pic="http://schemas.openxmlformats.org/drawingml/2006/picture" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:s="http://schemas.openxmlformats.org/officeDocument/2006/sharedTypes" xmlns:sl="http://schemas.openxmlformats.org/schemaLibrary/2006/main" xmlns:v="urn:schemas-microsoft-com:vml" xmlns:w="http://schemas.openxmlformats.org/wordprocessingml/2006/main" xmlns:w10="urn:schemas-microsoft-com:office:word" xmlns:w14="http://schemas.microsoft.com/office/word/2010/wordml" xmlns:w15="http://schemas.microsoft.com/office/word/2012/wordml" xmlns:wp="http://schemas.openxmlformats.org/drawingml/2006/wordprocessingDrawing" xmlns:wpg="http://schemas.microsoft.com/office/word/2010/wordprocessingGroup" xmlns:wps="http://schemas.microsoft.com/office/word/2010/wordprocessingShape" xmlns:x="urn:schemas-microsoft-com:office:excel" xmlns:x12ac="http://schemas.microsoft.com/office/spreadsheetml/2011/1/ac" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" mc:Ignorable="co co-ooxml w14 x14 w15">
   <numFmts>
     <numFmt co:extendedFormatCode="General" formatCode="General" numFmtId="1002"/>
+    <numFmt co:extendedFormatCode="dd.mm.yyyy" formatCode="dd.mm.yyyy" numFmtId="1003"/>
     <numFmt co:extendedFormatCode="General" formatCode="General" numFmtId="1001"/>
     <numFmt co:extendedFormatCode="General" formatCode="General" numFmtId="1000"/>
-    <numFmt co:extendedFormatCode="dd.mm.yyyy" formatCode="dd.mm.yyyy" numFmtId="1003"/>
   </numFmts>
   <fonts count="4">
     <font>
@@ -120,8 +120,8 @@
     <xf applyAlignment="true" applyBorder="false" applyFill="true" applyFont="true" applyNumberFormat="true" borderId="0" fillId="2" fontId="2" numFmtId="1001" quotePrefix="false">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf applyAlignment="true" applyBorder="false" applyFill="true" applyFont="true" applyNumberFormat="true" borderId="0" fillId="2" fontId="2" numFmtId="1002" quotePrefix="false">
-      <alignment horizontal="center" vertical="center"/>
+    <xf applyAlignment="true" applyBorder="false" applyFill="false" applyFont="true" applyNumberFormat="true" borderId="0" fillId="0" fontId="1" numFmtId="1002" quotePrefix="false">
+      <alignment shrinkToFit="false" vertical="bottom" wrapText="false"/>
     </xf>
     <xf applyAlignment="true" applyBorder="false" applyFill="true" applyFont="true" applyNumberFormat="true" borderId="0" fillId="3" fontId="3" numFmtId="1003" quotePrefix="false">
       <alignment horizontal="center"/>
@@ -378,7 +378,7 @@
   <dimension ref="A1:W300"/>
   <sheetFormatPr baseColWidth="8" customHeight="false" defaultColWidth="10.7884703773945" defaultRowHeight="15" zeroHeight="false"/>
   <cols>
-    <col customWidth="true" max="1" min="1" outlineLevel="0" width="71.0421201800537"/>
+    <col customWidth="true" max="1" min="1" outlineLevel="0" width="95.3880190081888"/>
     <col customWidth="true" max="2" min="2" outlineLevel="0" width="27.8048762828506"/>
   </cols>
   <sheetData>
@@ -386,12 +386,12 @@
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
     </row>
     <row outlineLevel="0" r="2">
-      <c r="A2" s="0" t="s">
+      <c r="A2" s="2" t="s">
         <v>2</v>
       </c>
       <c r="B2" s="3" t="n">
@@ -399,7 +399,7 @@
       </c>
     </row>
     <row outlineLevel="0" r="3">
-      <c r="A3" s="0" t="s">
+      <c r="A3" s="2" t="s">
         <v>3</v>
       </c>
       <c r="B3" s="3" t="n">
@@ -407,7 +407,7 @@
       </c>
     </row>
     <row outlineLevel="0" r="4">
-      <c r="A4" s="0" t="s">
+      <c r="A4" s="2" t="s">
         <v>4</v>
       </c>
       <c r="B4" s="3" t="n">
@@ -415,7 +415,7 @@
       </c>
     </row>
     <row outlineLevel="0" r="5">
-      <c r="A5" s="0" t="s">
+      <c r="A5" s="2" t="s">
         <v>5</v>
       </c>
       <c r="B5" s="3" t="n">
@@ -423,7 +423,7 @@
       </c>
     </row>
     <row outlineLevel="0" r="6">
-      <c r="A6" s="0" t="s">
+      <c r="A6" s="2" t="s">
         <v>6</v>
       </c>
       <c r="B6" s="3" t="n">
@@ -431,7 +431,7 @@
       </c>
     </row>
     <row outlineLevel="0" r="7">
-      <c r="A7" s="0" t="s">
+      <c r="A7" s="2" t="s">
         <v>7</v>
       </c>
       <c r="B7" s="3" t="n">
@@ -439,7 +439,7 @@
       </c>
     </row>
     <row outlineLevel="0" r="8">
-      <c r="A8" s="0" t="s">
+      <c r="A8" s="2" t="s">
         <v>8</v>
       </c>
       <c r="B8" s="3" t="n">
@@ -447,7 +447,7 @@
       </c>
     </row>
     <row outlineLevel="0" r="9">
-      <c r="A9" s="0" t="s">
+      <c r="A9" s="2" t="s">
         <v>9</v>
       </c>
       <c r="B9" s="3" t="n">
@@ -455,7 +455,7 @@
       </c>
     </row>
     <row outlineLevel="0" r="10">
-      <c r="A10" s="0" t="s">
+      <c r="A10" s="2" t="s">
         <v>10</v>
       </c>
       <c r="B10" s="3" t="n">
@@ -463,7 +463,7 @@
       </c>
     </row>
     <row outlineLevel="0" r="11">
-      <c r="A11" s="0" t="s">
+      <c r="A11" s="2" t="s">
         <v>11</v>
       </c>
       <c r="B11" s="3" t="n">

</xml_diff>